<commit_message>
France at the UK cuts, the UK host for the French-characteristics shocks, and the 2026-09-22 rebuild
The 2026-09-22 session per notes/TODO.md: D1 (France regrouped at the UK's income cuts, the hours typo
corrected, both variants re-swept), R5 (FRUK sweeps, UK shocks, six UK outputs), W6 (the UK paragraphs),
eight tables moved to appendix E; entries in the three research logs. Also the review memo
notes/esc_inequalityChannel.md (why inequality corners the chosen design, candidates, a pilot at rho = 1)
and results/diagnostics/thetaStakes.csv, the stakes decomposition it quotes.
</commit_message>
<xml_diff>
--- a/data/FRMain.xlsx
+++ b/data/FRMain.xlsx
@@ -1,22 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sxj477\Documents\GitHub\SSD\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sxj477\Documents\GitHub\SSDclaude\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB66E3A4-0BD1-4D86-B6AC-89398003BAA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B96B05A1-1992-4205-9564-D582A52BC61C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{D3C4F84A-0E01-44C3-A15D-A44758EFE8C0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="5" xr2:uid="{D3C4F84A-0E01-44C3-A15D-A44758EFE8C0}"/>
   </bookViews>
   <sheets>
     <sheet name="Readme" sheetId="4" r:id="rId1"/>
     <sheet name="population" sheetId="1" r:id="rId2"/>
     <sheet name="heterogeneity" sheetId="2" r:id="rId3"/>
-    <sheet name="calibration" sheetId="3" r:id="rId4"/>
+    <sheet name="heterogeneityUK" sheetId="5" r:id="rId4"/>
+    <sheet name="calibration" sheetId="3" r:id="rId5"/>
+    <sheet name="calibrationUK" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="25">
   <si>
     <t>t</t>
   </si>
@@ -108,6 +110,12 @@
   </si>
   <si>
     <t xml:space="preserve">Worker-to-retiree data is adjusted based on the retirement age in France relative to that of US/UK. This difference changes from 2,5 years in 2020 to an expected differencec of  2 years by 2050. </t>
+  </si>
+  <si>
+    <t>heterogeneityUK/calibrationUK (2026-09-22): France regrouped at the UK's own income cuts (cumulative shares 0.2924/0.8731/1), for the counterfactuals that impose French characteristics on the UK. Income, hours and group sizes are the LIS 2018 second sampling in calibration statistics AUG 2025.docx (SSD/Data). Voting shares have no CSES source at these cuts yet: they are the observed (US-cut) group values weighted by the population overlap of the new groups with the old, i.e. voting taken as flat within each observed group. Replace with CSES at the UK cuts when available.</t>
+  </si>
+  <si>
+    <t>2026-09-22: heterogeneity!C3 (low-group hours) corrected from 1731.91 to 1713.91, the value in calibration statistics AUG 2025.docx (SSD/Data); the workbook figure was a digit transposition. With it the average workweek is 35.24 at both the US and the UK cuts.</t>
   </si>
 </sst>
 </file>
@@ -503,7 +511,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05AA8116-F26D-48D0-B2CE-7FBA20E167F1}">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -524,6 +532,16 @@
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -711,7 +729,7 @@
         <v>0.58205409356725146</v>
       </c>
       <c r="C3">
-        <v>1731.91</v>
+        <v>1713.91</v>
       </c>
       <c r="D3" s="1">
         <v>25112</v>
@@ -772,6 +790,126 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34142F09-580B-4BFA-B78B-5C2D40A9041B}">
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <f>4800/(4800+9532+2084)</f>
+        <v>0.29239766081871343</v>
+      </c>
+      <c r="C3">
+        <v>1629.38</v>
+      </c>
+      <c r="D3" s="1">
+        <v>20011</v>
+      </c>
+      <c r="E3">
+        <v>0.80969999999999998</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <f>9532/(4800+9532+2084)</f>
+        <v>0.58065302144249509</v>
+      </c>
+      <c r="C4">
+        <v>1855.62</v>
+      </c>
+      <c r="D4" s="1">
+        <v>37081</v>
+      </c>
+      <c r="E4">
+        <v>0.83230000000000004</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <f>2084/(4800+9532+2084)</f>
+        <v>0.12694931773879142</v>
+      </c>
+      <c r="C5">
+        <v>2194.58</v>
+      </c>
+      <c r="D5" s="1">
+        <v>94604</v>
+      </c>
+      <c r="E5">
+        <v>0.8518</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11E48DC5-CA22-4A6E-BD10-69F2BD6158FF}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -836,7 +974,80 @@
       </c>
       <c r="H2">
         <f>SUMPRODUCT(heterogeneity!B3:B5,heterogeneity!C3:C5)/52</f>
-        <v>35.441714849021594</v>
+        <v>35.240234585863696</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6AAB2B7-DEB4-4692-8BCB-4698B5AA77FA}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2020</v>
+      </c>
+      <c r="B2">
+        <v>0.3</v>
+      </c>
+      <c r="C2">
+        <v>0.3</v>
+      </c>
+      <c r="D2">
+        <f>0.149/(1-B2)</f>
+        <v>0.21285714285714286</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2">
+        <f>SUMPRODUCT(heterogeneityUK!B3:B5,heterogeneityUK!C3:C5)/52</f>
+        <v>35.240359499175284</v>
       </c>
     </row>
   </sheetData>

</xml_diff>